<commit_message>
feat: add 4 provider columns to componente + Corrugadora del Plata
componente sheet now has 4 new columns:
- proveedor_insumo_id: 180/455 mapped (fleje 47/54, plástico 33/38,
  remache 15/17, cartón 84/84 = Corrugadora del Plata id=26)
- tallerista_id: 83/84 terminado mapped (from ruta_paso)
- proveedor_servicio_id: 58/84 procesado mapped (from ruta_paso)
- matriz_id: 72/79 crudo mapped (from ruta_paso)

proveedor_insumo expanded to 26 entries (+Corrugadora del Plata)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tdvjsW2k2dJPXLugCuJpZ
</commit_message>
<xml_diff>
--- a/Tablas_Supabase_Completas_v3.xlsx
+++ b/Tablas_Supabase_Completas_v3.xlsx
@@ -73787,7 +73787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="19.140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -74052,6 +74052,16 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>Szapiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Corrugadora del Plata</t>
         </is>
       </c>
     </row>
@@ -77309,7 +77319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H456"/>
+  <dimension ref="A1:K456"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -77359,6 +77369,21 @@
           <t>proveedor_insumo_id</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tallerista_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>proveedor_servicio_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>matriz_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -77387,6 +77412,9 @@
       </c>
       <c r="G2" t="n">
         <v>15000</v>
+      </c>
+      <c r="K2" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="3">
@@ -77417,6 +77445,9 @@
       <c r="G3" t="n">
         <v>3333</v>
       </c>
+      <c r="K3" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -77446,6 +77477,9 @@
       <c r="G4" t="n">
         <v>1146</v>
       </c>
+      <c r="K4" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -77475,6 +77509,9 @@
       <c r="G5" t="n">
         <v>769</v>
       </c>
+      <c r="K5" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -77504,6 +77541,9 @@
       <c r="G6" t="n">
         <v>757</v>
       </c>
+      <c r="K6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -77533,6 +77573,9 @@
       <c r="G7" t="n">
         <v>2381</v>
       </c>
+      <c r="K7" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -77562,6 +77605,9 @@
       <c r="G8" t="n">
         <v>1145</v>
       </c>
+      <c r="K8" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -77591,6 +77637,9 @@
       <c r="G9" t="n">
         <v>660</v>
       </c>
+      <c r="K9" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -77620,6 +77669,9 @@
       <c r="G10" t="n">
         <v>606</v>
       </c>
+      <c r="K10" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -77649,6 +77701,9 @@
       <c r="G11" t="n">
         <v>547</v>
       </c>
+      <c r="K11" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -77678,6 +77733,9 @@
       <c r="G12" t="n">
         <v>761</v>
       </c>
+      <c r="K12" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -77707,6 +77765,9 @@
       <c r="G13" t="n">
         <v>768</v>
       </c>
+      <c r="K13" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -77736,6 +77797,9 @@
       <c r="G14" t="n">
         <v>1334</v>
       </c>
+      <c r="K14" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -77765,6 +77829,9 @@
       <c r="G15" t="n">
         <v>990</v>
       </c>
+      <c r="K15" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -77794,6 +77861,9 @@
       <c r="G16" t="n">
         <v>1048</v>
       </c>
+      <c r="K16" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -77823,6 +77893,9 @@
       <c r="G17" t="n">
         <v>757</v>
       </c>
+      <c r="K17" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -77852,6 +77925,9 @@
       <c r="G18" t="n">
         <v>774</v>
       </c>
+      <c r="K18" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -77881,6 +77957,9 @@
       <c r="G19" t="n">
         <v>3439</v>
       </c>
+      <c r="K19" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -77910,6 +77989,9 @@
       <c r="G20" t="n">
         <v>3417</v>
       </c>
+      <c r="K20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -77968,6 +78050,9 @@
       <c r="G22" t="n">
         <v>839</v>
       </c>
+      <c r="K22" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -77997,6 +78082,9 @@
       <c r="G23" t="n">
         <v>844</v>
       </c>
+      <c r="K23" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -78055,6 +78143,9 @@
       <c r="G25" t="n">
         <v>1036</v>
       </c>
+      <c r="K25" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -78084,6 +78175,9 @@
       <c r="G26" t="n">
         <v>1043</v>
       </c>
+      <c r="K26" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -78113,6 +78207,9 @@
       <c r="G27" t="n">
         <v>960</v>
       </c>
+      <c r="K27" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -78142,6 +78239,9 @@
       <c r="G28" t="n">
         <v>1768</v>
       </c>
+      <c r="K28" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -78171,6 +78271,9 @@
       <c r="G29" t="n">
         <v>1768</v>
       </c>
+      <c r="K29" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -78200,6 +78303,9 @@
       <c r="G30" t="n">
         <v>1685</v>
       </c>
+      <c r="K30" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -78229,6 +78335,9 @@
       <c r="G31" t="n">
         <v>1685</v>
       </c>
+      <c r="K31" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -78258,6 +78367,9 @@
       <c r="G32" t="n">
         <v>1142</v>
       </c>
+      <c r="K32" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -78287,6 +78399,9 @@
       <c r="G33" t="n">
         <v>1149</v>
       </c>
+      <c r="K33" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -78316,6 +78431,9 @@
       <c r="G34" t="n">
         <v>6081</v>
       </c>
+      <c r="K34" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -78345,6 +78463,9 @@
       <c r="G35" t="n">
         <v>3094</v>
       </c>
+      <c r="K35" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -78374,6 +78495,9 @@
       <c r="G36" t="n">
         <v>976</v>
       </c>
+      <c r="K36" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -78403,6 +78527,9 @@
       <c r="G37" t="n">
         <v>957</v>
       </c>
+      <c r="K37" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -78432,6 +78559,9 @@
       <c r="G38" t="n">
         <v>2143</v>
       </c>
+      <c r="K38" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -78461,6 +78591,9 @@
       <c r="G39" t="n">
         <v>2150</v>
       </c>
+      <c r="K39" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -78490,6 +78623,9 @@
       <c r="G40" t="n">
         <v>17578</v>
       </c>
+      <c r="K40" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -78519,6 +78655,9 @@
       <c r="G41" t="n">
         <v>1235</v>
       </c>
+      <c r="K41" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -78548,6 +78687,9 @@
       <c r="G42" t="n">
         <v>1234</v>
       </c>
+      <c r="K42" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -78577,6 +78719,9 @@
       <c r="G43" t="n">
         <v>1235</v>
       </c>
+      <c r="K43" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -78606,6 +78751,9 @@
       <c r="G44" t="n">
         <v>8272</v>
       </c>
+      <c r="K44" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -78635,6 +78783,9 @@
       <c r="G45" t="n">
         <v>4945</v>
       </c>
+      <c r="K45" t="n">
+        <v>96</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -78664,6 +78815,9 @@
       <c r="G46" t="n">
         <v>9375</v>
       </c>
+      <c r="K46" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -78693,6 +78847,9 @@
       <c r="G47" t="n">
         <v>2144</v>
       </c>
+      <c r="K47" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -78722,6 +78879,9 @@
       <c r="G48" t="n">
         <v>1227</v>
       </c>
+      <c r="K48" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -78751,6 +78911,9 @@
       <c r="G49" t="n">
         <v>1829</v>
       </c>
+      <c r="K49" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -78780,6 +78943,9 @@
       <c r="G50" t="n">
         <v>4615</v>
       </c>
+      <c r="K50" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -78809,6 +78975,9 @@
       <c r="G51" t="n">
         <v>1668</v>
       </c>
+      <c r="K51" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -78838,6 +79007,9 @@
       <c r="G52" t="n">
         <v>756</v>
       </c>
+      <c r="K52" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -78867,6 +79039,9 @@
       <c r="G53" t="n">
         <v>1829</v>
       </c>
+      <c r="K53" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -78896,6 +79071,9 @@
       <c r="G54" t="n">
         <v>18868</v>
       </c>
+      <c r="K54" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -78925,6 +79103,9 @@
       <c r="G55" t="n">
         <v>945</v>
       </c>
+      <c r="K55" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -79012,6 +79193,9 @@
       <c r="G58" t="n">
         <v>913</v>
       </c>
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -79041,6 +79225,9 @@
       <c r="G59" t="n">
         <v>1429</v>
       </c>
+      <c r="K59" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -79070,6 +79257,9 @@
       <c r="G60" t="n">
         <v>1967</v>
       </c>
+      <c r="K60" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -79099,6 +79289,9 @@
       <c r="G61" t="n">
         <v>2810</v>
       </c>
+      <c r="K61" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -79128,6 +79321,9 @@
       <c r="G62" t="n">
         <v>7126</v>
       </c>
+      <c r="K62" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -79157,6 +79353,9 @@
       <c r="G63" t="n">
         <v>4261</v>
       </c>
+      <c r="K63" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -79186,6 +79385,9 @@
       <c r="G64" t="n">
         <v>180</v>
       </c>
+      <c r="K64" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -79215,6 +79417,9 @@
       <c r="G65" t="n">
         <v>1644</v>
       </c>
+      <c r="K65" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -79244,6 +79449,9 @@
       <c r="G66" t="n">
         <v>694</v>
       </c>
+      <c r="K66" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -79273,6 +79481,9 @@
       <c r="G67" t="n">
         <v>2198</v>
       </c>
+      <c r="K67" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -79302,6 +79513,9 @@
       <c r="G68" t="n">
         <v>954</v>
       </c>
+      <c r="K68" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -79331,6 +79545,9 @@
       <c r="G69" t="n">
         <v>2985</v>
       </c>
+      <c r="K69" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -79360,6 +79577,9 @@
       <c r="G70" t="n">
         <v>4004</v>
       </c>
+      <c r="K70" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -79418,6 +79638,9 @@
       <c r="G72" t="n">
         <v>300</v>
       </c>
+      <c r="K72" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -79447,6 +79670,9 @@
       <c r="G73" t="n">
         <v>252</v>
       </c>
+      <c r="K73" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -79476,6 +79702,9 @@
       <c r="G74" t="n">
         <v>410</v>
       </c>
+      <c r="K74" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -79505,6 +79734,9 @@
       <c r="G75" t="n">
         <v>1081</v>
       </c>
+      <c r="K75" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -79534,6 +79766,9 @@
       <c r="G76" t="n">
         <v>341</v>
       </c>
+      <c r="K76" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -79563,6 +79798,9 @@
       <c r="G77" t="n">
         <v>1071</v>
       </c>
+      <c r="K77" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -79650,6 +79888,9 @@
       <c r="G80" t="n">
         <v>5435</v>
       </c>
+      <c r="K80" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -79679,6 +79920,9 @@
       <c r="G81" t="n">
         <v>756</v>
       </c>
+      <c r="J81" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -79708,6 +79952,9 @@
       <c r="G82" t="n">
         <v>756</v>
       </c>
+      <c r="J82" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -79737,6 +79984,9 @@
       <c r="G83" t="n">
         <v>759</v>
       </c>
+      <c r="J83" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -79766,6 +80016,9 @@
       <c r="G84" t="n">
         <v>1676</v>
       </c>
+      <c r="J84" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -79795,6 +80048,9 @@
       <c r="G85" t="n">
         <v>769</v>
       </c>
+      <c r="J85" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -79824,6 +80080,9 @@
       <c r="G86" t="n">
         <v>1695</v>
       </c>
+      <c r="J86" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -79882,6 +80141,9 @@
       <c r="G88" t="n">
         <v>593</v>
       </c>
+      <c r="J88" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -79911,6 +80173,9 @@
       <c r="G89" t="n">
         <v>592</v>
       </c>
+      <c r="J89" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -79940,6 +80205,9 @@
       <c r="G90" t="n">
         <v>949</v>
       </c>
+      <c r="J90" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -79969,6 +80237,9 @@
       <c r="G91" t="n">
         <v>952</v>
       </c>
+      <c r="J91" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -79998,6 +80269,9 @@
       <c r="G92" t="n">
         <v>1299</v>
       </c>
+      <c r="J92" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -80027,6 +80301,9 @@
       <c r="G93" t="n">
         <v>833</v>
       </c>
+      <c r="J93" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -80056,6 +80333,9 @@
       <c r="G94" t="n">
         <v>2344</v>
       </c>
+      <c r="J94" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -80085,6 +80365,9 @@
       <c r="G95" t="n">
         <v>1007</v>
       </c>
+      <c r="J95" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -80114,6 +80397,9 @@
       <c r="G96" t="n">
         <v>765</v>
       </c>
+      <c r="J96" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -80143,6 +80429,9 @@
       <c r="G97" t="n">
         <v>1024</v>
       </c>
+      <c r="J97" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -80172,6 +80461,9 @@
       <c r="G98" t="n">
         <v>1020</v>
       </c>
+      <c r="J98" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -80201,6 +80493,9 @@
       <c r="G99" t="n">
         <v>719</v>
       </c>
+      <c r="J99" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -80230,6 +80525,9 @@
       <c r="G100" t="n">
         <v>722</v>
       </c>
+      <c r="J100" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -80259,6 +80557,9 @@
       <c r="G101" t="n">
         <v>826</v>
       </c>
+      <c r="J101" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -80289,6 +80590,9 @@
       <c r="G102" t="n">
         <v>545</v>
       </c>
+      <c r="J102" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -80318,6 +80622,9 @@
       <c r="G103" t="n">
         <v>2143</v>
       </c>
+      <c r="J103" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -80347,6 +80654,9 @@
       <c r="G104" t="n">
         <v>8108</v>
       </c>
+      <c r="J104" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -80405,6 +80715,9 @@
       <c r="G106" t="n">
         <v>652</v>
       </c>
+      <c r="J106" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -80492,6 +80805,9 @@
       <c r="G109" t="n">
         <v>1765</v>
       </c>
+      <c r="J109" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -80521,6 +80837,9 @@
       <c r="G110" t="n">
         <v>454</v>
       </c>
+      <c r="J110" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -80550,6 +80869,9 @@
       <c r="G111" t="n">
         <v>454</v>
       </c>
+      <c r="J111" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -80579,6 +80901,9 @@
       <c r="G112" t="n">
         <v>3125</v>
       </c>
+      <c r="J112" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -80608,6 +80933,9 @@
       <c r="G113" t="n">
         <v>2143</v>
       </c>
+      <c r="J113" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -80637,6 +80965,9 @@
       <c r="G114" t="n">
         <v>2098</v>
       </c>
+      <c r="J114" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -80666,6 +80997,9 @@
       <c r="G115" t="n">
         <v>1887</v>
       </c>
+      <c r="J115" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -80695,6 +81029,9 @@
       <c r="G116" t="n">
         <v>16667</v>
       </c>
+      <c r="J116" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -80724,6 +81061,9 @@
       <c r="G117" t="n">
         <v>60</v>
       </c>
+      <c r="J117" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -80840,6 +81180,9 @@
       <c r="G121" t="n">
         <v>1657</v>
       </c>
+      <c r="J121" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -80869,6 +81212,9 @@
       <c r="G122" t="n">
         <v>197</v>
       </c>
+      <c r="J122" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -80898,6 +81244,9 @@
       <c r="G123" t="n">
         <v>2362</v>
       </c>
+      <c r="J123" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -80927,6 +81276,9 @@
       <c r="G124" t="n">
         <v>9375</v>
       </c>
+      <c r="J124" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -80956,6 +81308,9 @@
       <c r="G125" t="n">
         <v>2143</v>
       </c>
+      <c r="J125" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -80985,6 +81340,9 @@
       <c r="G126" t="n">
         <v>6000</v>
       </c>
+      <c r="J126" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -81159,6 +81517,9 @@
       <c r="G132" t="n">
         <v>829</v>
       </c>
+      <c r="J132" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -81188,6 +81549,9 @@
       <c r="G133" t="n">
         <v>723</v>
       </c>
+      <c r="J133" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -81217,6 +81581,9 @@
       <c r="G134" t="n">
         <v>723</v>
       </c>
+      <c r="J134" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -81269,6 +81636,9 @@
       <c r="G136" t="n">
         <v>268</v>
       </c>
+      <c r="J136" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -81327,6 +81697,9 @@
       <c r="G138" t="n">
         <v>833</v>
       </c>
+      <c r="J138" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -81356,6 +81729,9 @@
       <c r="G139" t="n">
         <v>1333</v>
       </c>
+      <c r="J139" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -81443,6 +81819,9 @@
       <c r="G142" t="n">
         <v>754</v>
       </c>
+      <c r="J142" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -81472,6 +81851,9 @@
       <c r="G143" t="n">
         <v>759</v>
       </c>
+      <c r="J143" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -81501,6 +81883,9 @@
       <c r="G144" t="n">
         <v>829</v>
       </c>
+      <c r="J144" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -81530,6 +81915,9 @@
       <c r="G145" t="n">
         <v>754</v>
       </c>
+      <c r="J145" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -81559,6 +81947,9 @@
       <c r="G146" t="n">
         <v>1007</v>
       </c>
+      <c r="J146" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -81647,6 +82038,9 @@
       <c r="G149" t="n">
         <v>906</v>
       </c>
+      <c r="J149" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -81676,6 +82070,9 @@
       <c r="G150" t="n">
         <v>906</v>
       </c>
+      <c r="J150" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -81705,6 +82102,9 @@
       <c r="G151" t="n">
         <v>1667</v>
       </c>
+      <c r="J151" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -81735,6 +82135,9 @@
       <c r="G152" t="n">
         <v>20000</v>
       </c>
+      <c r="J152" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -81764,6 +82167,9 @@
       <c r="G153" t="n">
         <v>690</v>
       </c>
+      <c r="J153" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -81793,6 +82199,9 @@
       <c r="G154" t="n">
         <v>2222</v>
       </c>
+      <c r="J154" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -81910,6 +82319,9 @@
       <c r="G158" t="n">
         <v>2857</v>
       </c>
+      <c r="J158" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -81939,6 +82351,9 @@
       <c r="G159" t="n">
         <v>2857</v>
       </c>
+      <c r="J159" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -85669,6 +86084,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H289" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -85692,6 +86110,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H290" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -85715,6 +86136,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H291" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -85738,6 +86162,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H292" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -85761,6 +86188,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H293" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -85784,6 +86214,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H294" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -85807,6 +86240,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H295" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -85830,6 +86266,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H296" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -85853,6 +86292,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H297" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -85876,6 +86318,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H298" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -85899,6 +86344,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H299" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -85922,6 +86370,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H300" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -85945,6 +86396,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H301" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -85968,6 +86422,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H302" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -85991,6 +86448,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H303" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -86014,6 +86474,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H304" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -86037,6 +86500,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H305" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -86060,6 +86526,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H306" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -86083,6 +86552,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H307" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -86106,6 +86578,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H308" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -86129,6 +86604,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H309" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -86152,6 +86630,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H310" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -86175,6 +86656,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H311" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -86198,6 +86682,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H312" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -86221,6 +86708,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H313" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -86244,6 +86734,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H314" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -86267,6 +86760,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H315" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -86290,6 +86786,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H316" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -86313,6 +86812,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H317" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -86336,6 +86838,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H318" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -86359,6 +86864,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H319" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -86382,6 +86890,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H320" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -86405,6 +86916,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H321" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -86428,6 +86942,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H322" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -86451,6 +86968,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H323" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -86474,6 +86994,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H324" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -86497,6 +87020,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H325" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -86520,6 +87046,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H326" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -86543,6 +87072,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H327" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -86566,6 +87098,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H328" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -86589,6 +87124,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H329" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -86612,6 +87150,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H330" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -86635,6 +87176,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H331" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -86658,6 +87202,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H332" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -86681,6 +87228,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H333" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -86704,6 +87254,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H334" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -86727,6 +87280,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H335" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -86750,6 +87306,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H336" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -86773,6 +87332,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H337" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -86796,6 +87358,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H338" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -86819,6 +87384,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H339" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -86842,6 +87410,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H340" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -86865,6 +87436,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H341" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -86888,6 +87462,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H342" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -86911,6 +87488,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H343" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -86934,6 +87514,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H344" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -86957,6 +87540,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H345" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -86980,6 +87566,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H346" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -87003,6 +87592,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H347" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -87026,6 +87618,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H348" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -87049,6 +87644,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H349" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -87072,6 +87670,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H350" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -87095,6 +87696,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H351" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -87118,6 +87722,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H352" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -87141,6 +87748,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H353" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -87164,6 +87774,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H354" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -87187,6 +87800,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H355" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -87210,6 +87826,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H356" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -87233,6 +87852,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H357" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -87256,6 +87878,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H358" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -87279,6 +87904,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H359" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -87302,6 +87930,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H360" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -87325,6 +87956,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H361" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -87348,6 +87982,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H362" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -87371,6 +88008,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H363" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -87394,6 +88034,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H364" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -87417,6 +88060,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H365" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -87440,6 +88086,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H366" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -87463,6 +88112,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H367" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -87486,6 +88138,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H368" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -87509,6 +88164,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H369" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -87532,6 +88190,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H370" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -87555,6 +88216,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H371" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -87578,6 +88242,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="H372" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -87601,6 +88268,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I373" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -87624,6 +88294,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I374" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -87647,6 +88320,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I375" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -87670,6 +88346,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I376" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -87693,6 +88372,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I377" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -87716,6 +88398,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I378" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -87739,6 +88424,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I379" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -87762,6 +88450,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I380" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -87785,6 +88476,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I381" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -87808,6 +88502,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I382" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -87831,6 +88528,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I383" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -87854,6 +88554,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I384" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="n">
@@ -87877,6 +88580,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I385" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -87900,6 +88606,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I386" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -87923,6 +88632,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I387" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="n">
@@ -87946,6 +88658,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I388" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -87969,6 +88684,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I389" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -87992,6 +88710,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I390" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="n">
@@ -88015,6 +88736,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I391" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="n">
@@ -88061,6 +88785,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I393" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="n">
@@ -88084,6 +88811,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I394" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -88107,6 +88837,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I395" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="n">
@@ -88130,6 +88863,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I396" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="n">
@@ -88153,6 +88889,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I397" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -88176,6 +88915,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I398" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -88199,6 +88941,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I399" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -88222,6 +88967,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I400" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -88245,6 +88993,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I401" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="n">
@@ -88268,6 +89019,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I402" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -88291,6 +89045,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I403" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -88314,6 +89071,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I404" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -88337,6 +89097,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I405" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
@@ -88360,6 +89123,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I406" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
@@ -88383,6 +89149,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I407" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="n">
@@ -88406,6 +89175,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I408" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -88429,6 +89201,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I409" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -88452,6 +89227,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I410" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -88475,6 +89253,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I411" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -88498,6 +89279,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I412" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -88521,6 +89305,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I413" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -88544,6 +89331,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I414" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -88567,6 +89357,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I415" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -88590,6 +89383,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I416" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
@@ -88613,6 +89409,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I417" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="n">
@@ -88636,6 +89435,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I418" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -88659,6 +89461,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I419" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -88682,6 +89487,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I420" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="n">
@@ -88705,6 +89513,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I421" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -88728,6 +89539,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I422" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="n">
@@ -88751,6 +89565,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I423" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="n">
@@ -88774,6 +89591,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I424" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
@@ -88797,6 +89617,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I425" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -88820,6 +89643,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I426" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -88843,6 +89669,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I427" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="n">
@@ -88866,6 +89695,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I428" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="n">
@@ -88889,6 +89721,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I429" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="n">
@@ -88912,6 +89747,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I430" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="n">
@@ -88935,6 +89773,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I431" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="n">
@@ -88958,6 +89799,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I432" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="n">
@@ -88981,6 +89825,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I433" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="n">
@@ -89004,6 +89851,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I434" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="n">
@@ -89027,6 +89877,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I435" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="n">
@@ -89050,6 +89903,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I436" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="n">
@@ -89073,6 +89929,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I437" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
@@ -89096,6 +89955,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I438" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="n">
@@ -89119,6 +89981,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I439" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="n">
@@ -89142,6 +90007,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I440" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="n">
@@ -89165,6 +90033,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I441" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="n">
@@ -89188,6 +90059,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I442" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="n">
@@ -89211,6 +90085,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I443" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="n">
@@ -89234,6 +90111,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I444" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="n">
@@ -89257,6 +90137,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I445" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="n">
@@ -89280,6 +90163,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I446" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="n">
@@ -89303,6 +90189,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I447" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="n">
@@ -89326,6 +90215,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I448" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
@@ -89349,6 +90241,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I449" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="n">
@@ -89372,6 +90267,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I450" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="n">
@@ -89395,6 +90293,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I451" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="n">
@@ -89418,6 +90319,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I452" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="n">
@@ -89441,6 +90345,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I453" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="n">
@@ -89464,6 +90371,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I454" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="n">
@@ -89487,6 +90397,9 @@
           <t>unidad</t>
         </is>
       </c>
+      <c r="I455" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="n">
@@ -89509,6 +90422,9 @@
         <is>
           <t>unidad</t>
         </is>
+      </c>
+      <c r="I456" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(excel): corregir proveedor cartón a Gráfica Pol y agregar Corrugadora para cajas
- proveedor_insumo id=26: cambiado de 'Corrugadora del Plata' a 'Gráfica Pol' (verificado en codebase)
- proveedor_insumo id=27: 'Corrugadora' agregado para cajas
- Componentes de cartón (sector_id=10) apuntan correctamente a Gráfica Pol

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tdvjsW2k2dJPXLugCuJpZ
</commit_message>
<xml_diff>
--- a/Tablas_Supabase_Completas_v3.xlsx
+++ b/Tablas_Supabase_Completas_v3.xlsx
@@ -73787,7 +73787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="19.140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -74061,7 +74061,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Corrugadora del Plata</t>
+          <t>Gráfica Pol</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Corrugadora</t>
         </is>
       </c>
     </row>

</xml_diff>